<commit_message>
latest: new checklist and new Dockerfile
</commit_message>
<xml_diff>
--- a/dspackagefolder/template/checklist/GENERIC_CHECKLIST.xlsx
+++ b/dspackagefolder/template/checklist/GENERIC_CHECKLIST.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rajim\Desktop\NonPHD_Muizdeen\INTERVIEWS\dspackage\dspackagefolder\template\checklist\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA08DCA8-55E3-4CD3-B12D-BA820DC6E389}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5C3A037-56C9-47A5-BC42-466BA01EFB40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,32 +25,46 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
-  <si>
-    <t>check about 10 digits from the output of the analysis and ensure you can manually generate such numbers and they have been dq-ed</t>
-  </si>
-  <si>
-    <t>Spot-checking of high values within each column</t>
-  </si>
-  <si>
-    <t>Spot-checking of low values within each column</t>
-  </si>
-  <si>
-    <t>do you know the meaning of each column</t>
-  </si>
-  <si>
-    <t>CHECKLIST FOR TRANSFORMATION/EDA/PRE-PROCESSING</t>
-  </si>
-  <si>
-    <t>NULLS and different kind of values in each column</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+  <si>
+    <t>Checklist for Transformation / EDA / Pre-processing / Data Generation</t>
+  </si>
+  <si>
+    <t>Verify approximately 10 values from the analysis output. Manually reproduce these values where possible and confirm they have passed data quality (DQ) checks.</t>
+  </si>
+  <si>
+    <t>Perform spot checks on the highest values in each column.</t>
+  </si>
+  <si>
+    <t>Perform spot checks on the lowest values in each column.</t>
+  </si>
+  <si>
+    <t>Ensure you understand the meaning and business context of every column.</t>
+  </si>
+  <si>
+    <t>Review each column for null values and identify the different types of values it contains.</t>
+  </si>
+  <si>
+    <t>Consider carefully whether a pooled mean is more appropriate than a mean of means before aggregating data.</t>
+  </si>
+  <si>
+    <t>Before regenerating an existing dataset, investigate whether equivalent or complementary data is already available from other reliable sources.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -78,10 +92,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -111,10 +131,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{65C1E661-4582-4641-86AB-3C6FE5EE6E5A}" name="Table1" displayName="Table1" ref="A1:A1048576" totalsRowShown="0" headerRowDxfId="2" dataDxfId="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{65C1E661-4582-4641-86AB-3C6FE5EE6E5A}" name="Table1" displayName="Table1" ref="A1:A1048576" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0">
   <autoFilter ref="A1:A1048576" xr:uid="{65C1E661-4582-4641-86AB-3C6FE5EE6E5A}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{25BD2411-6041-4738-B1D5-AE3022ADC147}" name="CHECKLIST FOR TRANSFORMATION/EDA/PRE-PROCESSING" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{25BD2411-6041-4738-B1D5-AE3022ADC147}" name="Checklist for Transformation / EDA / Pre-processing / Data Generation" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -383,40 +403,53 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="69.453125" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A2" s="3"/>
+    </row>
+    <row r="3" spans="1:1" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A3" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A4" s="3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A5" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A6" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:1" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A2" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A3" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A4" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A5" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A6" s="1" t="s">
+    <row r="7" spans="1:1" ht="29" x14ac:dyDescent="0.35">
+      <c r="A7" s="3" t="s">
         <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" ht="29" x14ac:dyDescent="0.35">
+      <c r="A8" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" ht="29" x14ac:dyDescent="0.35">
+      <c r="A9" s="1" t="s">
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>